<commit_message>
Signed-off-by: Student Rani Wheeza (TL_KCOMP_B_Y3) <t00244793@mymtu.ie>
</commit_message>
<xml_diff>
--- a/Assignment 2.xlsx
+++ b/Assignment 2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StudentRaniWheeza(TL\Desktop\ere\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StudentRaniWheeza(TL\Desktop\awfe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{950E7557-5961-4F8F-958F-806BB9702CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83CC941E-16C6-47D9-BCF1-D274CA03663F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assignment generation" sheetId="1" r:id="rId1"/>
@@ -563,18 +563,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -583,10 +577,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1393,7 +1393,7 @@
   <cols>
     <col min="1" max="3" width="9.140625" customWidth="1"/>
     <col min="4" max="4" width="37.5703125" customWidth="1"/>
-    <col min="5" max="5" width="19" customWidth="1"/>
+    <col min="5" max="5" width="43.85546875" customWidth="1"/>
     <col min="6" max="6" width="21" customWidth="1"/>
     <col min="7" max="7" width="17.7109375" customWidth="1"/>
     <col min="8" max="8" width="27.5703125" customWidth="1"/>
@@ -1410,10 +1410,10 @@
     </row>
     <row r="2" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C2" s="4"/>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="47"/>
+      <c r="E2" s="41"/>
       <c r="F2" s="7"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -1425,7 +1425,7 @@
     <row r="3" spans="3:13" ht="408.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C3" s="4"/>
       <c r="D3" s="38"/>
-      <c r="E3" s="40"/>
+      <c r="E3" s="39"/>
       <c r="F3" s="5"/>
       <c r="G3" s="10"/>
       <c r="H3" s="6"/>
@@ -1445,10 +1445,10 @@
     </row>
     <row r="5" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C5" s="4"/>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="47"/>
+      <c r="E5" s="41"/>
       <c r="F5" s="7"/>
       <c r="H5" s="14"/>
       <c r="I5" s="11"/>
@@ -1458,7 +1458,7 @@
     <row r="6" spans="3:13" ht="138.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C6" s="4"/>
       <c r="D6" s="38"/>
-      <c r="E6" s="40"/>
+      <c r="E6" s="39"/>
       <c r="F6" s="15"/>
       <c r="G6" s="11"/>
       <c r="H6" s="14"/>
@@ -1478,10 +1478,10 @@
     </row>
     <row r="8" spans="3:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C8" s="4"/>
-      <c r="D8" s="46" t="s">
+      <c r="D8" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="47"/>
+      <c r="E8" s="41"/>
       <c r="F8" s="16"/>
       <c r="G8" s="11"/>
       <c r="H8" s="14"/>
@@ -1492,7 +1492,7 @@
     <row r="9" spans="3:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C9" s="4"/>
       <c r="D9" s="38"/>
-      <c r="E9" s="40"/>
+      <c r="E9" s="39"/>
       <c r="F9" s="16"/>
       <c r="G9" s="11"/>
       <c r="H9" s="14"/>
@@ -1512,16 +1512,16 @@
     </row>
     <row r="11" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C11" s="4"/>
-      <c r="D11" s="46" t="s">
+      <c r="D11" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="47"/>
+      <c r="E11" s="41"/>
       <c r="F11" s="17"/>
       <c r="G11" s="18"/>
-      <c r="H11" s="44" t="s">
+      <c r="H11" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="I11" s="45"/>
+      <c r="I11" s="43"/>
       <c r="J11" s="7"/>
       <c r="L11" s="14"/>
       <c r="M11" s="11"/>
@@ -1529,11 +1529,11 @@
     <row r="12" spans="3:13" ht="93" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C12" s="4"/>
       <c r="D12" s="38"/>
-      <c r="E12" s="40"/>
+      <c r="E12" s="39"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
       <c r="H12" s="38"/>
-      <c r="I12" s="40"/>
+      <c r="I12" s="39"/>
       <c r="J12" s="15"/>
       <c r="K12" s="11"/>
       <c r="L12" s="14"/>
@@ -1553,10 +1553,10 @@
     </row>
     <row r="14" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C14" s="4"/>
-      <c r="D14" s="46" t="s">
+      <c r="D14" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="47"/>
+      <c r="E14" s="41"/>
       <c r="F14" s="16"/>
       <c r="G14" s="11"/>
       <c r="H14" s="14"/>
@@ -1569,7 +1569,7 @@
     <row r="15" spans="3:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C15" s="4"/>
       <c r="D15" s="38"/>
-      <c r="E15" s="40"/>
+      <c r="E15" s="39"/>
       <c r="F15" s="16"/>
       <c r="G15" s="11"/>
       <c r="H15" s="14"/>
@@ -1593,10 +1593,10 @@
     </row>
     <row r="17" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C17" s="4"/>
-      <c r="D17" s="46" t="s">
+      <c r="D17" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="47"/>
+      <c r="E17" s="41"/>
       <c r="F17" s="17"/>
       <c r="G17" s="11"/>
       <c r="H17" s="14"/>
@@ -1609,7 +1609,7 @@
     <row r="18" spans="1:13" ht="107.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C18" s="4"/>
       <c r="D18" s="38"/>
-      <c r="E18" s="40"/>
+      <c r="E18" s="39"/>
       <c r="F18" s="19"/>
       <c r="H18" s="14"/>
       <c r="I18" s="11"/>
@@ -1630,18 +1630,18 @@
     </row>
     <row r="20" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C20" s="4"/>
-      <c r="D20" s="46" t="s">
+      <c r="D20" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="E20" s="47"/>
-      <c r="F20" s="41" t="s">
+      <c r="E20" s="41"/>
+      <c r="F20" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="G20" s="43"/>
-      <c r="H20" s="44" t="s">
+      <c r="G20" s="45"/>
+      <c r="H20" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="I20" s="45"/>
+      <c r="I20" s="43"/>
       <c r="J20" s="16"/>
       <c r="K20" s="11"/>
       <c r="L20" s="14"/>
@@ -1650,11 +1650,11 @@
     <row r="21" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C21" s="4"/>
       <c r="D21" s="38"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="43"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="44"/>
+      <c r="G21" s="45"/>
       <c r="H21" s="38"/>
-      <c r="I21" s="40"/>
+      <c r="I21" s="39"/>
       <c r="J21" s="16"/>
       <c r="K21" s="11"/>
       <c r="L21" s="14"/>
@@ -1672,25 +1672,25 @@
     </row>
     <row r="23" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C23" s="4"/>
-      <c r="D23" s="46" t="s">
+      <c r="D23" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="E23" s="47"/>
+      <c r="E23" s="41"/>
       <c r="F23" s="8"/>
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
       <c r="I23" s="21"/>
       <c r="J23" s="9"/>
       <c r="K23" s="17"/>
-      <c r="L23" s="44" t="s">
+      <c r="L23" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="M23" s="45"/>
+      <c r="M23" s="43"/>
     </row>
     <row r="24" spans="1:13" ht="113.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C24" s="4"/>
       <c r="D24" s="38"/>
-      <c r="E24" s="40"/>
+      <c r="E24" s="39"/>
       <c r="F24" s="5"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10"/>
@@ -1698,7 +1698,7 @@
       <c r="J24" s="6"/>
       <c r="K24" s="22"/>
       <c r="L24" s="38"/>
-      <c r="M24" s="40"/>
+      <c r="M24" s="39"/>
     </row>
     <row r="25" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D25" s="12"/>
@@ -1711,10 +1711,10 @@
     <row r="26" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="3"/>
       <c r="C26" s="23"/>
-      <c r="D26" s="44" t="s">
+      <c r="D26" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="E26" s="45"/>
+      <c r="E26" s="43"/>
       <c r="F26" s="11"/>
       <c r="J26" s="14"/>
       <c r="K26" s="11"/>
@@ -1726,7 +1726,7 @@
       <c r="B27" s="5"/>
       <c r="C27" s="6"/>
       <c r="D27" s="38"/>
-      <c r="E27" s="40"/>
+      <c r="E27" s="39"/>
       <c r="F27" s="11"/>
       <c r="J27" s="14"/>
       <c r="K27" s="11"/>
@@ -1744,15 +1744,15 @@
       <c r="M28" s="11"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="44" t="s">
+      <c r="A29" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="45"/>
+      <c r="B29" s="43"/>
       <c r="C29" s="24"/>
-      <c r="D29" s="46" t="s">
+      <c r="D29" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="47"/>
+      <c r="E29" s="41"/>
       <c r="F29" s="8"/>
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
@@ -1764,10 +1764,10 @@
     </row>
     <row r="30" spans="1:13" ht="322.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="38"/>
-      <c r="B30" s="40"/>
+      <c r="B30" s="39"/>
       <c r="C30" s="24"/>
       <c r="D30" s="38"/>
-      <c r="E30" s="40"/>
+      <c r="E30" s="39"/>
       <c r="F30" s="19"/>
       <c r="G30" s="20"/>
       <c r="H30" s="20"/>
@@ -1785,44 +1785,44 @@
       <c r="M31" s="7"/>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A32" s="46" t="s">
+      <c r="A32" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="B32" s="47"/>
+      <c r="B32" s="41"/>
       <c r="C32" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="46" t="s">
+      <c r="D32" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="E32" s="47"/>
-      <c r="F32" s="41" t="s">
+      <c r="E32" s="41"/>
+      <c r="F32" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="G32" s="42"/>
-      <c r="H32" s="42"/>
-      <c r="I32" s="42"/>
-      <c r="J32" s="42"/>
-      <c r="K32" s="43"/>
-      <c r="L32" s="46" t="s">
+      <c r="G32" s="47"/>
+      <c r="H32" s="47"/>
+      <c r="I32" s="47"/>
+      <c r="J32" s="47"/>
+      <c r="K32" s="45"/>
+      <c r="L32" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="M32" s="47"/>
+      <c r="M32" s="41"/>
     </row>
     <row r="33" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="48"/>
-      <c r="B33" s="39"/>
+      <c r="B33" s="46"/>
       <c r="C33" s="16"/>
       <c r="D33" s="38"/>
-      <c r="E33" s="40"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
-      <c r="I33" s="42"/>
-      <c r="J33" s="42"/>
-      <c r="K33" s="43"/>
+      <c r="E33" s="39"/>
+      <c r="F33" s="44"/>
+      <c r="G33" s="47"/>
+      <c r="H33" s="47"/>
+      <c r="I33" s="47"/>
+      <c r="J33" s="47"/>
+      <c r="K33" s="45"/>
       <c r="L33" s="38"/>
-      <c r="M33" s="39"/>
+      <c r="M33" s="46"/>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="20"/>
@@ -1834,33 +1834,46 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C35" s="4"/>
-      <c r="D35" s="44" t="s">
+      <c r="D35" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="E35" s="45"/>
+      <c r="E35" s="43"/>
       <c r="F35" s="11"/>
     </row>
     <row r="36" spans="1:13" ht="213.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C36" s="4"/>
       <c r="D36" s="38"/>
-      <c r="E36" s="40"/>
+      <c r="E36" s="39"/>
       <c r="F36" s="11"/>
     </row>
     <row r="38" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E38" s="25"/>
       <c r="F38" s="25"/>
       <c r="H38" s="38"/>
-      <c r="I38" s="39"/>
+      <c r="I38" s="46"/>
     </row>
     <row r="91" ht="0.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="F32:K32"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="F33:K33"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="L33:M33"/>
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="H11:I11"/>
@@ -1877,25 +1890,12 @@
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="D23:E23"/>
-    <mergeCell ref="L23:M23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="L32:M32"/>
-    <mergeCell ref="L33:M33"/>
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F32:K32"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="F33:K33"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D8:E8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>